<commit_message>
Finalize math course production audits
</commit_message>
<xml_diff>
--- a/Refined Courses/Math for College Readiness/mla_math_for_college_readiness_standards_crosswalk_v2.xlsx
+++ b/Refined Courses/Math for College Readiness/mla_math_for_college_readiness_standards_crosswalk_v2.xlsx
@@ -1,5 +1,19 @@
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="README" sheetId="1" r:id="rId1"/>
+    <sheet name="MLA Standards Crosswalk" sheetId="2" r:id="rId2"/>
+    <sheet name="Embedded Standards" sheetId="3" r:id="rId3"/>
+    <sheet name="Coverage Audit" sheetId="4" r:id="rId4"/>
+    <sheet name="MLA Inventory" sheetId="5" r:id="rId5"/>
+    <sheet name="Sources" sheetId="6" r:id="rId6"/>
+    <sheet name="Corrections Log" sheetId="7" r:id="rId7"/>
+  </sheets>
+</workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="2">
     <font>
@@ -51,21 +65,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheets>
-    <sheet name="README" sheetId="1" r:id="rId1"/>
-    <sheet name="MLA Standards Crosswalk" sheetId="2" r:id="rId2"/>
-    <sheet name="Embedded Standards" sheetId="3" r:id="rId3"/>
-    <sheet name="Coverage Audit" sheetId="4" r:id="rId4"/>
-    <sheet name="MLA Inventory" sheetId="5" r:id="rId5"/>
-    <sheet name="Sources" sheetId="6" r:id="rId6"/>
-    <sheet name="Corrections Log" sheetId="7" r:id="rId7"/>
-  </sheets>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -73,12 +73,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A" t="inlineStr" s="1">
+      <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Item</t>
         </is>
       </c>
-      <c r="B" t="inlineStr" s="1">
+      <c r="B1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Detail</t>
         </is>
@@ -172,7 +172,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -197,97 +197,97 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A" t="inlineStr" s="1">
+      <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">MLA Standard Code</t>
         </is>
       </c>
-      <c r="B" t="inlineStr" s="1">
+      <c r="B1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">MLA Standard Statement</t>
         </is>
       </c>
-      <c r="C" t="inlineStr" s="1">
+      <c r="C1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Florida B.E.S.T. Benchmark Code</t>
         </is>
       </c>
-      <c r="D" t="inlineStr" s="1">
+      <c r="D1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Florida B.E.S.T. Benchmark Description</t>
         </is>
       </c>
-      <c r="E" t="inlineStr" s="1">
+      <c r="E1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Benchmark Inclusion Rationale</t>
         </is>
       </c>
-      <c r="F" t="inlineStr" s="1">
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Common Core Standard Code</t>
         </is>
       </c>
-      <c r="G" t="inlineStr" s="1">
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Common Core Description</t>
         </is>
       </c>
-      <c r="H" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Common Core Alignment Type: Primary or Support</t>
         </is>
       </c>
-      <c r="I" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">SAT Primary Domain</t>
         </is>
       </c>
-      <c r="J" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">SAT Skill Connection</t>
         </is>
       </c>
-      <c r="K" t="inlineStr" s="1">
+      <c r="K1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">SAT Support Domain(s)</t>
         </is>
       </c>
-      <c r="L" t="inlineStr" s="1">
+      <c r="L1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">SAT Alignment Type: Primary or Support</t>
         </is>
       </c>
-      <c r="M" t="inlineStr" s="1">
+      <c r="M1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">ACT Primary Reporting Category</t>
         </is>
       </c>
-      <c r="N" t="inlineStr" s="1">
+      <c r="N1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">ACT Skill Connection</t>
         </is>
       </c>
-      <c r="O" t="inlineStr" s="1">
+      <c r="O1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">ACT Support Category(s)</t>
         </is>
       </c>
-      <c r="P" t="inlineStr" s="1">
+      <c r="P1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">ACT Alignment Type: Primary or Support</t>
         </is>
       </c>
-      <c r="Q" t="inlineStr" s="1">
+      <c r="Q1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Course Domain</t>
         </is>
       </c>
-      <c r="R" t="inlineStr" s="1">
+      <c r="R1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">DOK Level</t>
         </is>
       </c>
-      <c r="S" t="inlineStr" s="1">
+      <c r="S1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Notes</t>
         </is>
@@ -5244,7 +5244,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -5254,22 +5254,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A" t="inlineStr" s="1">
+      <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Embedded Standard Code</t>
         </is>
       </c>
-      <c r="B" t="inlineStr" s="1">
+      <c r="B1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Embedded Standard</t>
         </is>
       </c>
-      <c r="C" t="inlineStr" s="1">
+      <c r="C1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Role</t>
         </is>
       </c>
-      <c r="D" t="inlineStr" s="1">
+      <c r="D1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Where Embedded</t>
         </is>
@@ -5433,7 +5433,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -5442,17 +5442,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A" t="inlineStr" s="1">
+      <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Audit Area</t>
         </is>
       </c>
-      <c r="B" t="inlineStr" s="1">
+      <c r="B1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Result</t>
         </is>
       </c>
-      <c r="C" t="inlineStr" s="1">
+      <c r="C1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Notes</t>
         </is>
@@ -5598,7 +5598,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -5608,22 +5608,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A" t="inlineStr" s="1">
+      <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">MLA Domain</t>
         </is>
       </c>
-      <c r="B" t="inlineStr" s="1">
+      <c r="B1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Domain Name</t>
         </is>
       </c>
-      <c r="C" t="inlineStr" s="1">
+      <c r="C1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Main Crosswalk Standards</t>
         </is>
       </c>
-      <c r="D" t="inlineStr" s="1">
+      <c r="D1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Role</t>
         </is>
@@ -5787,7 +5787,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
@@ -5796,17 +5796,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A" t="inlineStr" s="1">
+      <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Source</t>
         </is>
       </c>
-      <c r="B" t="inlineStr" s="1">
+      <c r="B1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Use</t>
         </is>
       </c>
-      <c r="C" t="inlineStr" s="1">
+      <c r="C1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Location</t>
         </is>
@@ -5935,7 +5935,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="48" customWidth="1"/>
@@ -5946,27 +5946,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A" t="inlineStr" s="1">
+      <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Issue</t>
         </is>
       </c>
-      <c r="B" t="inlineStr" s="1">
+      <c r="B1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Location</t>
         </is>
       </c>
-      <c r="C" t="inlineStr" s="1">
+      <c r="C1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Correction Made</t>
         </is>
       </c>
-      <c r="D" t="inlineStr" s="1">
+      <c r="D1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Rationale</t>
         </is>
       </c>
-      <c r="E" t="inlineStr" s="1">
+      <c r="E1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Date</t>
         </is>

</xml_diff>